<commit_message>
Round-2 residual audit: 16 fact fixes (9 eps), Nina->Ingrid (Ep 195), comment mining results
- Fact spot-check of 19 episodes vs full source chapters (two agents):
  fixed 16 confirmed mismatches across Eps 61, 195, 400, 479, 927, 975,
  1067, 1193, 1194 (number inflation, item/color, creature, sword-exchange
  continuity, disciple-count line, Nina drift-name)
- Ruled canon (documented in LS Localization Issues): Union of Seven
  Divine Kingdoms (Ep 740 bridge), hundred-thousand-worlds cosmology,
  Elder Apeiron female, Steel Longsword
- Listener-comment mining (1,927 comments): all cited names except Nina
  are absent from our text (earlier aired-version artifacts); no
  duplicated-episode content found
- Regenerated 9 docx, refreshed word counts, updated all three zips,
  appended log rows F1-F16, added FTP_Residual_Audit_Round2.md

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EjoRUNGYsE63Le6qUWSN6W
</commit_message>
<xml_diff>
--- a/FTP_Remaster_Corrections_Log.xlsx
+++ b/FTP_Remaster_Corrections_Log.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1647"/>
+  <dimension ref="A1:G1663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50598,6 +50598,534 @@
         </is>
       </c>
     </row>
+    <row r="1648">
+      <c r="A1648" t="n">
+        <v>1647</v>
+      </c>
+      <c r="B1648" t="n">
+        <v>195</v>
+      </c>
+      <c r="C1648" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D1648" t="inlineStr">
+        <is>
+          <t>Fact Fix — Name Drift</t>
+        </is>
+      </c>
+      <c r="E1648" t="inlineStr">
+        <is>
+          <t>"And Nina! You’re here too!"</t>
+        </is>
+      </c>
+      <c r="F1648" t="inlineStr">
+        <is>
+          <t>"And Ingrid! You’re here too!"</t>
+        </is>
+      </c>
+      <c r="G1648" t="inlineStr">
+        <is>
+          <t>Residual drift-name "Nina" for Ingrid (source ch 183: Zhu Qianning); surfaced by listener comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" t="n">
+        <v>1648</v>
+      </c>
+      <c r="B1649" t="n">
+        <v>927</v>
+      </c>
+      <c r="C1649" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="D1649" t="inlineStr">
+        <is>
+          <t>Fact Fix — Number</t>
+        </is>
+      </c>
+      <c r="E1649" t="inlineStr">
+        <is>
+          <t>putting thousands of feet between them in an instant</t>
+        </is>
+      </c>
+      <c r="F1649" t="inlineStr">
+        <is>
+          <t>putting several hundred feet between them in an instant</t>
+        </is>
+      </c>
+      <c r="G1649" t="inlineStr">
+        <is>
+          <t>Priest retreat distance conformed to source (several hundred feet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" t="n">
+        <v>1649</v>
+      </c>
+      <c r="B1650" t="n">
+        <v>927</v>
+      </c>
+      <c r="C1650" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="D1650" t="inlineStr">
+        <is>
+          <t>Fact Fix — Time</t>
+        </is>
+      </c>
+      <c r="E1650" t="inlineStr">
+        <is>
+          <t>One hundred and twenty thousand years. That was how long</t>
+        </is>
+      </c>
+      <c r="F1650" t="inlineStr">
+        <is>
+          <t>One hundred thousand years. That was how long</t>
+        </is>
+      </c>
+      <c r="G1650" t="inlineStr">
+        <is>
+          <t>Brianna’s seal duration conformed to source (past hundred thousand years)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" t="n">
+        <v>1650</v>
+      </c>
+      <c r="B1651" t="n">
+        <v>975</v>
+      </c>
+      <c r="C1651" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="D1651" t="inlineStr">
+        <is>
+          <t>Fact Fix — Creature</t>
+        </is>
+      </c>
+      <c r="E1651" t="inlineStr">
+        <is>
+          <t>the water churned with countless piranhas</t>
+        </is>
+      </c>
+      <c r="F1651" t="inlineStr">
+        <is>
+          <t>the water churned with countless koi fish</t>
+        </is>
+      </c>
+      <c r="G1651" t="inlineStr">
+        <is>
+          <t>Pond fish conformed to source (countless koi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" t="n">
+        <v>1651</v>
+      </c>
+      <c r="B1652" t="n">
+        <v>1067</v>
+      </c>
+      <c r="C1652" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="D1652" t="inlineStr">
+        <is>
+          <t>Fact Fix — Number</t>
+        </is>
+      </c>
+      <c r="E1652" t="inlineStr">
+        <is>
+          <t>ten thousand feet high and a hundred thousand feet wide</t>
+        </is>
+      </c>
+      <c r="F1652" t="inlineStr">
+        <is>
+          <t>ten thousand feet high and tens of thousands of feet wide</t>
+        </is>
+      </c>
+      <c r="G1652" t="inlineStr">
+        <is>
+          <t>Rock width conformed to source (tens of thousands of feet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" t="n">
+        <v>1652</v>
+      </c>
+      <c r="B1653" t="n">
+        <v>1193</v>
+      </c>
+      <c r="C1653" t="inlineStr">
+        <is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="D1653" t="inlineStr">
+        <is>
+          <t>Fact Fix — Number</t>
+        </is>
+      </c>
+      <c r="E1653" t="inlineStr">
+        <is>
+          <t>At thirty feet out, he made his move</t>
+        </is>
+      </c>
+      <c r="F1653" t="inlineStr">
+        <is>
+          <t>At three hundred feet out, he made his move</t>
+        </is>
+      </c>
+      <c r="G1653" t="inlineStr">
+        <is>
+          <t>Distance conformed to source (thirty zhang ≈ 300 ft)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="n">
+        <v>1653</v>
+      </c>
+      <c r="B1654" t="n">
+        <v>1193</v>
+      </c>
+      <c r="C1654" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="D1654" t="inlineStr">
+        <is>
+          <t>Fact Fix — Lore</t>
+        </is>
+      </c>
+      <c r="E1654" t="inlineStr">
+        <is>
+          <t>the origin of all primates</t>
+        </is>
+      </c>
+      <c r="F1654" t="inlineStr">
+        <is>
+          <t>the origin of all living creatures</t>
+        </is>
+      </c>
+      <c r="G1654" t="inlineStr">
+        <is>
+          <t>Sacred Race lore conformed to source</t>
+        </is>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="n">
+        <v>1654</v>
+      </c>
+      <c r="B1655" t="n">
+        <v>1193</v>
+      </c>
+      <c r="C1655" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+      <c r="D1655" t="inlineStr">
+        <is>
+          <t>Fact Fix — Continuity</t>
+        </is>
+      </c>
+      <c r="E1655" t="inlineStr">
+        <is>
+          <t>A violent tremor ripped up the blade and tore it straight from Zane’s grasp… (first exchange)</t>
+        </is>
+      </c>
+      <c r="F1655" t="inlineStr">
+        <is>
+          <t>…fighting to tear it from Zane’s grasp — but he flooded his grip with the power of his Dragon Scales…</t>
+        </is>
+      </c>
+      <c r="G1655" t="inlineStr">
+        <is>
+          <t>First exchange: Zane keeps his sword (source: dragon-scale power suppresses the vibration); removed stray WEAPON CLATTER SFX; sword is lost only on the second exchange</t>
+        </is>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" t="n">
+        <v>1655</v>
+      </c>
+      <c r="B1656" t="n">
+        <v>1193</v>
+      </c>
+      <c r="C1656" t="inlineStr">
+        <is>
+          <t>F9</t>
+        </is>
+      </c>
+      <c r="D1656" t="inlineStr">
+        <is>
+          <t>Fact Fix — Continuity</t>
+        </is>
+      </c>
+      <c r="E1656" t="inlineStr">
+        <is>
+          <t>And the Master of the Elysian Keep, as far as Zane knew, had never taken on anyone else.</t>
+        </is>
+      </c>
+      <c r="F1656" t="inlineStr">
+        <is>
+          <t>Zane had never heard of the Master of the Elysian Keep taking on anyone else.</t>
+        </is>
+      </c>
+      <c r="G1656" t="inlineStr">
+        <is>
+          <t>Master has two prior disciples (source + Ep 1194); reframed as Zane’s knowledge gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" t="n">
+        <v>1656</v>
+      </c>
+      <c r="B1657" t="n">
+        <v>1194</v>
+      </c>
+      <c r="C1657" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="D1657" t="inlineStr">
+        <is>
+          <t>Fact Fix — Time</t>
+        </is>
+      </c>
+      <c r="E1657" t="inlineStr">
+        <is>
+          <t>the first disciple, who’d joined a few hundred years before him</t>
+        </is>
+      </c>
+      <c r="F1657" t="inlineStr">
+        <is>
+          <t>the first disciple, who’d joined a hundred years before him</t>
+        </is>
+      </c>
+      <c r="G1657" t="inlineStr">
+        <is>
+          <t>Conformed to source (a hundred years earlier than Xian An)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" t="n">
+        <v>1657</v>
+      </c>
+      <c r="B1658" t="n">
+        <v>61</v>
+      </c>
+      <c r="C1658" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="D1658" t="inlineStr">
+        <is>
+          <t>Fact Fix — Count</t>
+        </is>
+      </c>
+      <c r="E1658" t="inlineStr">
+        <is>
+          <t>Julian had sent his friends to plead for its return</t>
+        </is>
+      </c>
+      <c r="F1658" t="inlineStr">
+        <is>
+          <t>Julian had sent a friend to plead for its return</t>
+        </is>
+      </c>
+      <c r="G1658" t="inlineStr">
+        <is>
+          <t>Source: He Bing sent one person to intercede</t>
+        </is>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" t="n">
+        <v>1658</v>
+      </c>
+      <c r="B1659" t="n">
+        <v>400</v>
+      </c>
+      <c r="C1659" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="D1659" t="inlineStr">
+        <is>
+          <t>Fact Fix — Item</t>
+        </is>
+      </c>
+      <c r="E1659" t="inlineStr">
+        <is>
+          <t>Evil Jace’s ring had been bigger, but it had always been more than enough</t>
+        </is>
+      </c>
+      <c r="F1659" t="inlineStr">
+        <is>
+          <t>Evil Jace’s ring hadn’t held much space, but it had always been more than enough</t>
+        </is>
+      </c>
+      <c r="G1659" t="inlineStr">
+        <is>
+          <t>Ring comparison conformed to source (didn’t have much space, but enough)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" t="n">
+        <v>1659</v>
+      </c>
+      <c r="B1660" t="n">
+        <v>400</v>
+      </c>
+      <c r="C1660" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="D1660" t="inlineStr">
+        <is>
+          <t>Fact Fix — Color</t>
+        </is>
+      </c>
+      <c r="E1660" t="inlineStr">
+        <is>
+          <t>the blue stone carving back at Cloud Hall</t>
+        </is>
+      </c>
+      <c r="F1660" t="inlineStr">
+        <is>
+          <t>the green stone carving back at Cloud Hall</t>
+        </is>
+      </c>
+      <c r="G1660" t="inlineStr">
+        <is>
+          <t>Cloud Hall stone color conformed to source (green stone, faint green light)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" t="n">
+        <v>1660</v>
+      </c>
+      <c r="B1661" t="n">
+        <v>479</v>
+      </c>
+      <c r="C1661" t="inlineStr">
+        <is>
+          <t>F14</t>
+        </is>
+      </c>
+      <c r="D1661" t="inlineStr">
+        <is>
+          <t>Fact Fix — Number</t>
+        </is>
+      </c>
+      <c r="E1661" t="inlineStr">
+        <is>
+          <t>engineered to accommodate a hundred thousand spectators</t>
+        </is>
+      </c>
+      <c r="F1661" t="inlineStr">
+        <is>
+          <t>engineered to accommodate hundreds of thousands of spectators</t>
+        </is>
+      </c>
+      <c r="G1661" t="inlineStr">
+        <is>
+          <t>Capacity conformed to source</t>
+        </is>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" t="n">
+        <v>1661</v>
+      </c>
+      <c r="B1662" t="n">
+        <v>479</v>
+      </c>
+      <c r="C1662" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="D1662" t="inlineStr">
+        <is>
+          <t>Fact Fix — Number</t>
+        </is>
+      </c>
+      <c r="E1662" t="inlineStr">
+        <is>
+          <t>Millions of cultivators had flooded the city to watch…</t>
+        </is>
+      </c>
+      <c r="F1662" t="inlineStr">
+        <is>
+          <t>Hundreds of thousands of cultivators had flooded the city to watch, and even they were just a fraction of all who’d wanted to come.</t>
+        </is>
+      </c>
+      <c r="G1662" t="inlineStr">
+        <is>
+          <t>Crowd size conformed to source (hundreds of thousands; “millions” was sect-population figure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" t="n">
+        <v>1662</v>
+      </c>
+      <c r="B1663" t="n">
+        <v>479</v>
+      </c>
+      <c r="C1663" t="inlineStr">
+        <is>
+          <t>F16</t>
+        </is>
+      </c>
+      <c r="D1663" t="inlineStr">
+        <is>
+          <t>Fact Fix — Number</t>
+        </is>
+      </c>
+      <c r="E1663" t="inlineStr">
+        <is>
+          <t>tens of thousands of cultivators were lining up to pay</t>
+        </is>
+      </c>
+      <c r="F1663" t="inlineStr">
+        <is>
+          <t>hundreds of thousands of cultivators were lining up to pay</t>
+        </is>
+      </c>
+      <c r="G1663" t="inlineStr">
+        <is>
+          <t>Ticket queue conformed to source</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>